<commit_message>
add validation step to Cross validation Process
</commit_message>
<xml_diff>
--- a/estimation/notsensor/DenseModel/Dense_1st_torch_optimized/IWALQQ_1st_correction/angle/0_fold/0.xlsx
+++ b/estimation/notsensor/DenseModel/Dense_1st_torch_optimized/IWALQQ_1st_correction/angle/0_fold/0.xlsx
@@ -426,13 +426,13 @@
         <v>-12.84196021680824</v>
       </c>
       <c r="E2">
-        <v>-11.9440469963205</v>
+        <v>-26.02628337423908</v>
       </c>
       <c r="F2">
-        <v>0.1479827190582071</v>
+        <v>-2.503795294457598</v>
       </c>
       <c r="G2">
-        <v>-7.173082660792168</v>
+        <v>-15.00566622415806</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -449,13 +449,13 @@
         <v>-12.71643442446966</v>
       </c>
       <c r="E3">
-        <v>-11.97914266987994</v>
+        <v>-25.09397925943594</v>
       </c>
       <c r="F3">
-        <v>0.3341905991661052</v>
+        <v>-2.578330964994095</v>
       </c>
       <c r="G3">
-        <v>-6.47609033459063</v>
+        <v>-14.96536529803575</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -472,13 +472,13 @@
         <v>-12.47310014886157</v>
       </c>
       <c r="E4">
-        <v>-13.3015838773919</v>
+        <v>-25.72777995307547</v>
       </c>
       <c r="F4">
-        <v>0.3125859489336913</v>
+        <v>-2.661308527732521</v>
       </c>
       <c r="G4">
-        <v>-7.354457519252218</v>
+        <v>-14.84633628844402</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -495,13 +495,13 @@
         <v>-12.11331913943963</v>
       </c>
       <c r="E5">
-        <v>-13.2610223357052</v>
+        <v>-26.53846736992862</v>
       </c>
       <c r="F5">
-        <v>0.5872336464340758</v>
+        <v>-2.50573698764976</v>
       </c>
       <c r="G5">
-        <v>-7.433457067455847</v>
+        <v>-14.6117708948045</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -518,13 +518,13 @@
         <v>-11.64090941610433</v>
       </c>
       <c r="E6">
-        <v>-14.16743716460649</v>
+        <v>-26.34218066406615</v>
       </c>
       <c r="F6">
-        <v>0.5711508933087234</v>
+        <v>-2.745197294614028</v>
       </c>
       <c r="G6">
-        <v>-7.818102732572688</v>
+        <v>-14.50911418817724</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -541,13 +541,13 @@
         <v>-11.07914292675722</v>
       </c>
       <c r="E7">
-        <v>-14.27495672297061</v>
+        <v>-27.5569891013638</v>
       </c>
       <c r="F7">
-        <v>1.089144769259907</v>
+        <v>-2.593297078860473</v>
       </c>
       <c r="G7">
-        <v>-6.938239181327348</v>
+        <v>-14.53244029204694</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -564,13 +564,13 @@
         <v>-10.44983419553826</v>
       </c>
       <c r="E8">
-        <v>-15.67276079491822</v>
+        <v>-26.89474053400808</v>
       </c>
       <c r="F8">
-        <v>0.8753315454537158</v>
+        <v>-2.212557054613945</v>
       </c>
       <c r="G8">
-        <v>-6.419347584047522</v>
+        <v>-14.12312113102591</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -587,13 +587,13 @@
         <v>-9.763522020068494</v>
       </c>
       <c r="E9">
-        <v>-14.7661512416346</v>
+        <v>-28.1653850558203</v>
       </c>
       <c r="F9">
-        <v>1.127178430192044</v>
+        <v>-2.267593784855944</v>
       </c>
       <c r="G9">
-        <v>-6.227620649686171</v>
+        <v>-14.139524884173</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -610,13 +610,13 @@
         <v>-9.032633399222496</v>
       </c>
       <c r="E10">
-        <v>-16.35251644278759</v>
+        <v>-28.01354985081712</v>
       </c>
       <c r="F10">
-        <v>1.604891284447296</v>
+        <v>-2.295153568347084</v>
       </c>
       <c r="G10">
-        <v>-5.665013298560268</v>
+        <v>-13.5365172905586</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -633,13 +633,13 @@
         <v>-8.275057976045334</v>
       </c>
       <c r="E11">
-        <v>-16.10650256384689</v>
+        <v>-28.77333721982406</v>
       </c>
       <c r="F11">
-        <v>1.169128612204617</v>
+        <v>-2.276364538916785</v>
       </c>
       <c r="G11">
-        <v>-5.038946099992076</v>
+        <v>-13.28149603603193</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -656,13 +656,13 @@
         <v>-7.495862978727758</v>
       </c>
       <c r="E12">
-        <v>-18.66139061491638</v>
+        <v>-29.70793274247508</v>
       </c>
       <c r="F12">
-        <v>1.487369144277325</v>
+        <v>-2.220115078797088</v>
       </c>
       <c r="G12">
-        <v>-5.145644982722786</v>
+        <v>-13.32729081247667</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -679,13 +679,13 @@
         <v>-6.6939160579045</v>
       </c>
       <c r="E13">
-        <v>-18.94482780305647</v>
+        <v>-29.71454431452628</v>
       </c>
       <c r="F13">
-        <v>1.288488071273997</v>
+        <v>-2.189866414716461</v>
       </c>
       <c r="G13">
-        <v>-4.61912257797494</v>
+        <v>-12.96470993337907</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -702,13 +702,13 @@
         <v>-5.88600134966678</v>
       </c>
       <c r="E14">
-        <v>-18.62038528277692</v>
+        <v>-29.82550777737323</v>
       </c>
       <c r="F14">
-        <v>1.486878750774868</v>
+        <v>-2.248962973599581</v>
       </c>
       <c r="G14">
-        <v>-3.423899769204167</v>
+        <v>-12.8721603222832</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -725,13 +725,13 @@
         <v>-5.076858783042178</v>
       </c>
       <c r="E15">
-        <v>-20.16281975758151</v>
+        <v>-31.29294392989978</v>
       </c>
       <c r="F15">
-        <v>1.592715940360949</v>
+        <v>-1.707985215690322</v>
       </c>
       <c r="G15">
-        <v>-3.513744664594447</v>
+        <v>-11.76365063282256</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -748,13 +748,13 @@
         <v>-4.2692650412097</v>
       </c>
       <c r="E16">
-        <v>-21.63139482132099</v>
+        <v>-31.48354513664562</v>
       </c>
       <c r="F16">
-        <v>2.038768592481205</v>
+        <v>-1.854414893115787</v>
       </c>
       <c r="G16">
-        <v>-3.11077844046328</v>
+        <v>-11.75409308785068</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -771,13 +771,13 @@
         <v>-3.479964770861568</v>
       </c>
       <c r="E17">
-        <v>-21.3589980528116</v>
+        <v>-32.7938907900831</v>
       </c>
       <c r="F17">
-        <v>2.121330314783426</v>
+        <v>-1.849283157055444</v>
       </c>
       <c r="G17">
-        <v>-1.556424341046829</v>
+        <v>-11.66193743167399</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -794,13 +794,13 @@
         <v>-2.720937044912232</v>
       </c>
       <c r="E18">
-        <v>-22.12244895729074</v>
+        <v>-32.91942461804972</v>
       </c>
       <c r="F18">
-        <v>2.020789706370844</v>
+        <v>-1.747663185917015</v>
       </c>
       <c r="G18">
-        <v>-1.33707090416026</v>
+        <v>-11.08289984303669</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -817,13 +817,13 @@
         <v>-2.001365747441979</v>
       </c>
       <c r="E19">
-        <v>-23.29347610788223</v>
+        <v>-33.77973052460491</v>
       </c>
       <c r="F19">
-        <v>2.218570707463254</v>
+        <v>-1.644550496718741</v>
       </c>
       <c r="G19">
-        <v>-0.8192287498163818</v>
+        <v>-10.73679885963358</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -840,13 +840,13 @@
         <v>-1.335721915267748</v>
       </c>
       <c r="E20">
-        <v>-24.88704611118143</v>
+        <v>-34.88161014133629</v>
       </c>
       <c r="F20">
-        <v>2.141530882268095</v>
+        <v>-1.320213180561428</v>
       </c>
       <c r="G20">
-        <v>-0.9020288042990935</v>
+        <v>-10.73261764061748</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -863,13 +863,13 @@
         <v>-0.7372717129417363</v>
       </c>
       <c r="E21">
-        <v>-24.63066655523717</v>
+        <v>-34.60625401506289</v>
       </c>
       <c r="F21">
-        <v>2.224742044614111</v>
+        <v>-1.37343081598688</v>
       </c>
       <c r="G21">
-        <v>-0.3546499626538384</v>
+        <v>-10.48804446781274</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -886,13 +886,13 @@
         <v>-0.2117656691844344</v>
       </c>
       <c r="E22">
-        <v>-26.55582501080002</v>
+        <v>-35.55253526489071</v>
       </c>
       <c r="F22">
-        <v>2.304585065100344</v>
+        <v>-1.123847030993</v>
       </c>
       <c r="G22">
-        <v>0.5201716277351907</v>
+        <v>-10.38813882452862</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -909,13 +909,13 @@
         <v>0.237784578365794</v>
       </c>
       <c r="E23">
-        <v>-25.64557456441423</v>
+        <v>-36.18034025894409</v>
       </c>
       <c r="F23">
-        <v>2.388624594849159</v>
+        <v>-1.117104120334212</v>
       </c>
       <c r="G23">
-        <v>0.5768647200952097</v>
+        <v>-10.03933312541993</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -932,13 +932,13 @@
         <v>0.6076276132382472</v>
       </c>
       <c r="E24">
-        <v>-26.3365427139266</v>
+        <v>-36.30487329415502</v>
       </c>
       <c r="F24">
-        <v>2.711167667212008</v>
+        <v>-0.8463754290164718</v>
       </c>
       <c r="G24">
-        <v>0.6836331242822448</v>
+        <v>-9.711777818127818</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -955,13 +955,13 @@
         <v>0.9024407677695094</v>
       </c>
       <c r="E25">
-        <v>-26.15440296086409</v>
+        <v>-36.57081245872947</v>
       </c>
       <c r="F25">
-        <v>2.556229828192389</v>
+        <v>-0.7446055233781358</v>
       </c>
       <c r="G25">
-        <v>1.179450219153351</v>
+        <v>-10.56179349079109</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -978,13 +978,13 @@
         <v>1.130750603553288</v>
       </c>
       <c r="E26">
-        <v>-27.98649221862129</v>
+        <v>-36.30356003669279</v>
       </c>
       <c r="F26">
-        <v>2.645511266866119</v>
+        <v>-0.8013246678152207</v>
       </c>
       <c r="G26">
-        <v>1.347135971808515</v>
+        <v>-10.12590389127187</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1001,13 +1001,13 @@
         <v>1.29672882835036</v>
       </c>
       <c r="E27">
-        <v>-27.21297904489711</v>
+        <v>-36.64360994263977</v>
       </c>
       <c r="F27">
-        <v>2.652822437563228</v>
+        <v>-0.8439234615041853</v>
       </c>
       <c r="G27">
-        <v>1.102297955360636</v>
+        <v>-10.21538462665283</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1024,13 +1024,13 @@
         <v>1.409879374076198</v>
       </c>
       <c r="E28">
-        <v>-26.98657798688363</v>
+        <v>-36.64420090849777</v>
       </c>
       <c r="F28">
-        <v>2.866579332386029</v>
+        <v>-0.7979681230990772</v>
       </c>
       <c r="G28">
-        <v>0.9248063668181508</v>
+        <v>-10.58236853131766</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -1047,13 +1047,13 @@
         <v>1.479280467169327</v>
       </c>
       <c r="E29">
-        <v>-27.08542551752306</v>
+        <v>-36.6011170067888</v>
       </c>
       <c r="F29">
-        <v>2.543749644901811</v>
+        <v>-0.8712065702827898</v>
       </c>
       <c r="G29">
-        <v>1.288893544136117</v>
+        <v>-10.19198569078126</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -1070,13 +1070,13 @@
         <v>1.50872235312339</v>
       </c>
       <c r="E30">
-        <v>-26.05114016806718</v>
+        <v>-36.36010029891556</v>
       </c>
       <c r="F30">
-        <v>2.340768153254626</v>
+        <v>-0.7429355346940919</v>
       </c>
       <c r="G30">
-        <v>0.9336587655901619</v>
+        <v>-10.12933692699609</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -1093,13 +1093,13 @@
         <v>1.499645910311893</v>
       </c>
       <c r="E31">
-        <v>-25.50822594776159</v>
+        <v>-36.60007092929303</v>
       </c>
       <c r="F31">
-        <v>2.637194458142012</v>
+        <v>-0.645024164417996</v>
       </c>
       <c r="G31">
-        <v>1.42042813950244</v>
+        <v>-10.39531608725776</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -1116,13 +1116,13 @@
         <v>1.451615924292997</v>
       </c>
       <c r="E32">
-        <v>-25.23044029518308</v>
+        <v>-35.98650345751976</v>
       </c>
       <c r="F32">
-        <v>2.527836707094033</v>
+        <v>-0.7829523071885305</v>
       </c>
       <c r="G32">
-        <v>-0.05896527726829302</v>
+        <v>-10.5855168601255</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -1139,13 +1139,13 @@
         <v>1.359559092444083</v>
       </c>
       <c r="E33">
-        <v>-25.02278259108734</v>
+        <v>-35.3862791344101</v>
       </c>
       <c r="F33">
-        <v>2.51149633170641</v>
+        <v>-0.7491085285797539</v>
       </c>
       <c r="G33">
-        <v>-0.05047041741452316</v>
+        <v>-10.44727178895108</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -1162,13 +1162,13 @@
         <v>1.216953358123502</v>
       </c>
       <c r="E34">
-        <v>-26.03906725636273</v>
+        <v>-35.31745538644152</v>
       </c>
       <c r="F34">
-        <v>2.580537441260137</v>
+        <v>-0.6380178329251178</v>
       </c>
       <c r="G34">
-        <v>0.2440787508510522</v>
+        <v>-11.13881826774051</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -1185,13 +1185,13 @@
         <v>1.019270275049161</v>
       </c>
       <c r="E35">
-        <v>-24.22769576719062</v>
+        <v>-34.83921683191348</v>
       </c>
       <c r="F35">
-        <v>2.489107217543545</v>
+        <v>-0.6694966225989017</v>
       </c>
       <c r="G35">
-        <v>-0.8750180632441799</v>
+        <v>-11.37380079011798</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -1208,13 +1208,13 @@
         <v>0.762320144015299</v>
       </c>
       <c r="E36">
-        <v>-24.38555837109801</v>
+        <v>-34.55411090110157</v>
       </c>
       <c r="F36">
-        <v>2.817934285024031</v>
+        <v>-0.7657951615417471</v>
       </c>
       <c r="G36">
-        <v>-0.881831165964</v>
+        <v>-11.18483816128192</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -1231,13 +1231,13 @@
         <v>0.4426645192216139</v>
       </c>
       <c r="E37">
-        <v>-23.15826493096121</v>
+        <v>-34.30779135016535</v>
       </c>
       <c r="F37">
-        <v>2.953905823989153</v>
+        <v>-0.4598956470359457</v>
       </c>
       <c r="G37">
-        <v>-1.319101262973095</v>
+        <v>-11.10847049678202</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -1254,13 +1254,13 @@
         <v>0.06096766954741774</v>
       </c>
       <c r="E38">
-        <v>-22.57178679070183</v>
+        <v>-33.39753411106855</v>
       </c>
       <c r="F38">
-        <v>3.312517669804698</v>
+        <v>-0.7718422435821835</v>
       </c>
       <c r="G38">
-        <v>-1.166015016146117</v>
+        <v>-11.14234399873984</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -1277,13 +1277,13 @@
         <v>-0.3792131950306627</v>
       </c>
       <c r="E39">
-        <v>-21.32061470712259</v>
+        <v>-33.26571476117928</v>
       </c>
       <c r="F39">
-        <v>3.23153978597663</v>
+        <v>-0.4906860633980033</v>
       </c>
       <c r="G39">
-        <v>-2.078573515137299</v>
+        <v>-11.38472890094312</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -1300,13 +1300,13 @@
         <v>-0.8761753799626675</v>
       </c>
       <c r="E40">
-        <v>-22.73367067952803</v>
+        <v>-32.80679694100495</v>
       </c>
       <c r="F40">
-        <v>2.9415217313173</v>
+        <v>-0.5665429799419652</v>
       </c>
       <c r="G40">
-        <v>-1.952544357002784</v>
+        <v>-10.97097360889947</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -1323,13 +1323,13 @@
         <v>-1.425366338744107</v>
       </c>
       <c r="E41">
-        <v>-22.03943297178213</v>
+        <v>-32.45478733520372</v>
       </c>
       <c r="F41">
-        <v>3.710447146026719</v>
+        <v>-0.4936814399265263</v>
       </c>
       <c r="G41">
-        <v>-1.707083957993522</v>
+        <v>-10.87555706536659</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -1346,13 +1346,13 @@
         <v>-2.015231157067686</v>
       </c>
       <c r="E42">
-        <v>-19.35638910629557</v>
+        <v>-31.92914471476338</v>
       </c>
       <c r="F42">
-        <v>3.629187617281699</v>
+        <v>-0.4005795707910843</v>
       </c>
       <c r="G42">
-        <v>-1.975105724852917</v>
+        <v>-11.1638029549254</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -1369,13 +1369,13 @@
         <v>-2.642726177895209</v>
       </c>
       <c r="E43">
-        <v>-19.06090617729508</v>
+        <v>-30.76484461231028</v>
       </c>
       <c r="F43">
-        <v>3.626334719946457</v>
+        <v>-0.2707893093856522</v>
       </c>
       <c r="G43">
-        <v>-1.99534971082556</v>
+        <v>-11.83455258663713</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -1392,13 +1392,13 @@
         <v>-3.302493342235638</v>
       </c>
       <c r="E44">
-        <v>-18.21863718271244</v>
+        <v>-30.2375196637761</v>
       </c>
       <c r="F44">
-        <v>3.052082271834144</v>
+        <v>-0.3805165122952803</v>
       </c>
       <c r="G44">
-        <v>-3.409508827744955</v>
+        <v>-11.33185948868096</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -1415,13 +1415,13 @@
         <v>-3.981372365049176</v>
       </c>
       <c r="E45">
-        <v>-19.16474408629096</v>
+        <v>-30.19498370742205</v>
       </c>
       <c r="F45">
-        <v>3.732410479344545</v>
+        <v>-0.1880801376857327</v>
       </c>
       <c r="G45">
-        <v>-2.769391673908096</v>
+        <v>-11.62516389182377</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -1438,13 +1438,13 @@
         <v>-4.675719094584311</v>
       </c>
       <c r="E46">
-        <v>-18.47992560448101</v>
+        <v>-29.83686292594746</v>
       </c>
       <c r="F46">
-        <v>3.417352534833392</v>
+        <v>-0.2017366026882854</v>
       </c>
       <c r="G46">
-        <v>-3.775936560759186</v>
+        <v>-11.51028134051998</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -1461,13 +1461,13 @@
         <v>-5.382159326199743</v>
       </c>
       <c r="E47">
-        <v>-16.87972591523458</v>
+        <v>-29.11895035608946</v>
       </c>
       <c r="F47">
-        <v>3.637928550116039</v>
+        <v>-0.4617975785927733</v>
       </c>
       <c r="G47">
-        <v>-2.914674964899012</v>
+        <v>-12.02274385836254</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -1484,13 +1484,13 @@
         <v>-6.0910658296472</v>
       </c>
       <c r="E48">
-        <v>-16.91935459127571</v>
+        <v>-28.33362239367926</v>
       </c>
       <c r="F48">
-        <v>3.645466693481515</v>
+        <v>-0.2823317807762605</v>
       </c>
       <c r="G48">
-        <v>-3.595746877602195</v>
+        <v>-11.80071881122578</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -1507,13 +1507,13 @@
         <v>-6.795857888023868</v>
       </c>
       <c r="E49">
-        <v>-15.47371171991107</v>
+        <v>-28.04341513689771</v>
       </c>
       <c r="F49">
-        <v>3.430016615687391</v>
+        <v>-0.2600337870277034</v>
       </c>
       <c r="G49">
-        <v>-3.723262470683842</v>
+        <v>-11.22059867419713</v>
       </c>
     </row>
     <row r="50" spans="1:7">
@@ -1530,13 +1530,13 @@
         <v>-7.495637586243294</v>
       </c>
       <c r="E50">
-        <v>-15.16670382456106</v>
+        <v>-28.32056680311515</v>
       </c>
       <c r="F50">
-        <v>3.807939362396998</v>
+        <v>-0.1487823880969242</v>
       </c>
       <c r="G50">
-        <v>-3.488435543946719</v>
+        <v>-11.71292976461539</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -1553,13 +1553,13 @@
         <v>-8.181818297857365</v>
       </c>
       <c r="E51">
-        <v>-15.69483710570561</v>
+        <v>-27.07734671989338</v>
       </c>
       <c r="F51">
-        <v>3.742847908619819</v>
+        <v>-0.3388628858129099</v>
       </c>
       <c r="G51">
-        <v>-3.68121192124402</v>
+        <v>-12.02276041109024</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -1576,13 +1576,13 @@
         <v>-8.840007259460936</v>
       </c>
       <c r="E52">
-        <v>-14.42420616931541</v>
+        <v>-27.24917966611443</v>
       </c>
       <c r="F52">
-        <v>3.924293504529023</v>
+        <v>-0.2514999460440628</v>
       </c>
       <c r="G52">
-        <v>-3.827829362087262</v>
+        <v>-12.41833749757775</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -1599,13 +1599,13 @@
         <v>-9.46911285745356</v>
       </c>
       <c r="E53">
-        <v>-14.41931994586113</v>
+        <v>-26.42154217105057</v>
       </c>
       <c r="F53">
-        <v>3.839377562068045</v>
+        <v>-0.05480244951451464</v>
       </c>
       <c r="G53">
-        <v>-3.518664135265804</v>
+        <v>-11.92355991400598</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -1622,13 +1622,13 @@
         <v>-10.06146960155995</v>
       </c>
       <c r="E54">
-        <v>-13.30257108472558</v>
+        <v>-25.73400660483602</v>
       </c>
       <c r="F54">
-        <v>4.046996254436102</v>
+        <v>-0.08581901017753653</v>
       </c>
       <c r="G54">
-        <v>-5.115158168851638</v>
+        <v>-11.89134830590887</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -1645,13 +1645,13 @@
         <v>-10.59765823125841</v>
       </c>
       <c r="E55">
-        <v>-12.36365539787123</v>
+        <v>-24.95343354013388</v>
       </c>
       <c r="F55">
-        <v>3.84201839734817</v>
+        <v>-0.2674236526280778</v>
       </c>
       <c r="G55">
-        <v>-4.351696709312613</v>
+        <v>-12.25976898733774</v>
       </c>
     </row>
     <row r="56" spans="1:7">
@@ -1668,13 +1668,13 @@
         <v>-11.07769205788198</v>
       </c>
       <c r="E56">
-        <v>-11.79041851561028</v>
+        <v>-25.72057515092927</v>
       </c>
       <c r="F56">
-        <v>3.659481013202077</v>
+        <v>0.09423989869938081</v>
       </c>
       <c r="G56">
-        <v>-4.095877613310972</v>
+        <v>-12.20689626453004</v>
       </c>
     </row>
     <row r="57" spans="1:7">
@@ -1691,13 +1691,13 @@
         <v>-11.49666896398776</v>
       </c>
       <c r="E57">
-        <v>-12.44283123742134</v>
+        <v>-24.80376294570637</v>
       </c>
       <c r="F57">
-        <v>3.72862152684414</v>
+        <v>-0.2917204969195901</v>
       </c>
       <c r="G57">
-        <v>-3.998329078450806</v>
+        <v>-12.21457673018115</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -1714,13 +1714,13 @@
         <v>-11.83854448409222</v>
       </c>
       <c r="E58">
-        <v>-10.04166223654223</v>
+        <v>-24.38332583341223</v>
       </c>
       <c r="F58">
-        <v>3.633281408986334</v>
+        <v>-0.2988983004648478</v>
       </c>
       <c r="G58">
-        <v>-4.618092998312226</v>
+        <v>-12.38696345750208</v>
       </c>
     </row>
     <row r="59" spans="1:7">
@@ -1737,13 +1737,13 @@
         <v>-12.10150994821576</v>
       </c>
       <c r="E59">
-        <v>-9.440724678776357</v>
+        <v>-23.81850738433154</v>
       </c>
       <c r="F59">
-        <v>3.605302471589378</v>
+        <v>-0.2478849506982458</v>
       </c>
       <c r="G59">
-        <v>-4.182716533351594</v>
+        <v>-12.09647632861319</v>
       </c>
     </row>
     <row r="60" spans="1:7">
@@ -1760,13 +1760,13 @@
         <v>-12.28712958082474</v>
       </c>
       <c r="E60">
-        <v>-11.38911873447256</v>
+        <v>-23.59544834013571</v>
       </c>
       <c r="F60">
-        <v>3.617550712007171</v>
+        <v>-0.2626539131227582</v>
       </c>
       <c r="G60">
-        <v>-5.264241966121637</v>
+        <v>-12.69121252419772</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -1783,13 +1783,13 @@
         <v>-12.38736964106221</v>
       </c>
       <c r="E61">
-        <v>-10.36827389587144</v>
+        <v>-23.74756883900138</v>
       </c>
       <c r="F61">
-        <v>3.482901247416917</v>
+        <v>-0.2460641991468925</v>
       </c>
       <c r="G61">
-        <v>-4.799507583318748</v>
+        <v>-12.38953906193163</v>
       </c>
     </row>
     <row r="62" spans="1:7">
@@ -1806,13 +1806,13 @@
         <v>-12.39736177962232</v>
       </c>
       <c r="E62">
-        <v>-8.696945465386539</v>
+        <v>-23.46269159612685</v>
       </c>
       <c r="F62">
-        <v>3.182878171266575</v>
+        <v>-0.4506709476383704</v>
       </c>
       <c r="G62">
-        <v>-4.149700462688442</v>
+        <v>-12.38317950395069</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -1829,13 +1829,13 @@
         <v>-12.32800270523627</v>
       </c>
       <c r="E63">
-        <v>-8.886987405592434</v>
+        <v>-23.16023481715455</v>
       </c>
       <c r="F63">
-        <v>2.775150765404242</v>
+        <v>-0.4582728752938615</v>
       </c>
       <c r="G63">
-        <v>-4.268363656998079</v>
+        <v>-12.36756366064195</v>
       </c>
     </row>
     <row r="64" spans="1:7">
@@ -1852,13 +1852,13 @@
         <v>-12.17997317808846</v>
       </c>
       <c r="E64">
-        <v>-8.551459180942112</v>
+        <v>-23.23048050596153</v>
       </c>
       <c r="F64">
-        <v>2.603807938339581</v>
+        <v>-0.3460025844576389</v>
       </c>
       <c r="G64">
-        <v>-4.547780321603645</v>
+        <v>-12.5497396711225</v>
       </c>
     </row>
     <row r="65" spans="1:7">
@@ -1875,13 +1875,13 @@
         <v>-11.94819266677478</v>
       </c>
       <c r="E65">
-        <v>-7.577339137152142</v>
+        <v>-23.43329274286906</v>
       </c>
       <c r="F65">
-        <v>2.670551156717943</v>
+        <v>-0.3264506286493621</v>
       </c>
       <c r="G65">
-        <v>-3.786255531205094</v>
+        <v>-12.31697521425635</v>
       </c>
     </row>
     <row r="66" spans="1:7">
@@ -1898,13 +1898,13 @@
         <v>-11.64998234250278</v>
       </c>
       <c r="E66">
-        <v>-9.232500915429666</v>
+        <v>-22.75023583744809</v>
       </c>
       <c r="F66">
-        <v>2.406446091152988</v>
+        <v>-0.6836617051867734</v>
       </c>
       <c r="G66">
-        <v>-3.854019087848436</v>
+        <v>-12.70949004612003</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -1921,13 +1921,13 @@
         <v>-11.29298322148002</v>
       </c>
       <c r="E67">
-        <v>-8.766602452572524</v>
+        <v>-22.96122649841347</v>
       </c>
       <c r="F67">
-        <v>2.596799950111897</v>
+        <v>-0.8257209161950689</v>
       </c>
       <c r="G67">
-        <v>-4.559400336446487</v>
+        <v>-13.00729348065071</v>
       </c>
     </row>
     <row r="68" spans="1:7">
@@ -1944,13 +1944,13 @@
         <v>-10.87554726009174</v>
       </c>
       <c r="E68">
-        <v>-7.308230040772324</v>
+        <v>-22.96254881282371</v>
       </c>
       <c r="F68">
-        <v>2.364312011576994</v>
+        <v>-0.9418447721891149</v>
       </c>
       <c r="G68">
-        <v>-4.288763238611067</v>
+        <v>-12.24622885608212</v>
       </c>
     </row>
     <row r="69" spans="1:7">
@@ -1967,13 +1967,13 @@
         <v>-10.41495874253121</v>
       </c>
       <c r="E69">
-        <v>-7.159564767574514</v>
+        <v>-22.72667418718618</v>
       </c>
       <c r="F69">
-        <v>2.162102558349217</v>
+        <v>-0.9517321655089297</v>
       </c>
       <c r="G69">
-        <v>-4.555424371253823</v>
+        <v>-12.77493622088589</v>
       </c>
     </row>
     <row r="70" spans="1:7">
@@ -1990,13 +1990,13 @@
         <v>-9.922722033799174</v>
       </c>
       <c r="E70">
-        <v>-8.703860445196252</v>
+        <v>-22.59648508793967</v>
       </c>
       <c r="F70">
-        <v>2.266582882129514</v>
+        <v>-1.183661784414346</v>
       </c>
       <c r="G70">
-        <v>-3.762323597501703</v>
+        <v>-12.09394376127565</v>
       </c>
     </row>
     <row r="71" spans="1:7">
@@ -2013,13 +2013,13 @@
         <v>-9.399462252112382</v>
       </c>
       <c r="E71">
-        <v>-7.611655913182268</v>
+        <v>-22.25548646668808</v>
       </c>
       <c r="F71">
-        <v>2.270383431773558</v>
+        <v>-1.274046608468606</v>
       </c>
       <c r="G71">
-        <v>-3.665559661934345</v>
+        <v>-11.77799853718976</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -2036,13 +2036,13 @@
         <v>-8.852653682454916</v>
       </c>
       <c r="E72">
-        <v>-7.439044069431898</v>
+        <v>-22.89106232213862</v>
       </c>
       <c r="F72">
-        <v>1.640194646419806</v>
+        <v>-1.126684189347588</v>
       </c>
       <c r="G72">
-        <v>-3.478421143690424</v>
+        <v>-12.20274484042379</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -2059,13 +2059,13 @@
         <v>-8.291983786485041</v>
       </c>
       <c r="E73">
-        <v>-8.408006181327131</v>
+        <v>-22.60603563962184</v>
       </c>
       <c r="F73">
-        <v>1.724167906776397</v>
+        <v>-1.254619736138152</v>
       </c>
       <c r="G73">
-        <v>-2.691749449375568</v>
+        <v>-12.28667048038986</v>
       </c>
     </row>
     <row r="74" spans="1:7">
@@ -2082,13 +2082,13 @@
         <v>-7.715098658134549</v>
       </c>
       <c r="E74">
-        <v>-7.471318503684564</v>
+        <v>-22.46916704121401</v>
       </c>
       <c r="F74">
-        <v>1.629435810592246</v>
+        <v>-1.477613755869571</v>
       </c>
       <c r="G74">
-        <v>-2.249192411140257</v>
+        <v>-11.96780535513833</v>
       </c>
     </row>
     <row r="75" spans="1:7">
@@ -2105,13 +2105,13 @@
         <v>-7.116864474413036</v>
       </c>
       <c r="E75">
-        <v>-9.131230651196134</v>
+        <v>-22.67473711879221</v>
       </c>
       <c r="F75">
-        <v>1.344614933018081</v>
+        <v>-1.328485257445784</v>
       </c>
       <c r="G75">
-        <v>-2.137130444635927</v>
+        <v>-11.47522928435018</v>
       </c>
     </row>
     <row r="76" spans="1:7">
@@ -2128,13 +2128,13 @@
         <v>-6.504877870053117</v>
       </c>
       <c r="E76">
-        <v>-8.322907097774991</v>
+        <v>-22.65620660315282</v>
       </c>
       <c r="F76">
-        <v>1.447244684020522</v>
+        <v>-1.762995438175431</v>
       </c>
       <c r="G76">
-        <v>-2.594343267973592</v>
+        <v>-11.46896904273541</v>
       </c>
     </row>
     <row r="77" spans="1:7">
@@ -2151,13 +2151,13 @@
         <v>-5.87483546953774</v>
       </c>
       <c r="E77">
-        <v>-8.862334393094676</v>
+        <v>-22.85213103109468</v>
       </c>
       <c r="F77">
-        <v>1.426956309591157</v>
+        <v>-1.706277122105749</v>
       </c>
       <c r="G77">
-        <v>-2.327255074956271</v>
+        <v>-11.58173284489407</v>
       </c>
     </row>
     <row r="78" spans="1:7">
@@ -2174,13 +2174,13 @@
         <v>-5.218958315315596</v>
       </c>
       <c r="E78">
-        <v>-9.632958400401963</v>
+        <v>-23.39230099615162</v>
       </c>
       <c r="F78">
-        <v>1.16164348435292</v>
+        <v>-1.605756394510835</v>
       </c>
       <c r="G78">
-        <v>-1.534409213210676</v>
+        <v>-11.18703636352</v>
       </c>
     </row>
     <row r="79" spans="1:7">
@@ -2197,13 +2197,13 @@
         <v>-4.541025940919487</v>
       </c>
       <c r="E79">
-        <v>-10.29023923177127</v>
+        <v>-23.69525590726477</v>
       </c>
       <c r="F79">
-        <v>1.277982715871694</v>
+        <v>-1.980116333021001</v>
       </c>
       <c r="G79">
-        <v>-0.7082559527944724</v>
+        <v>-11.62562405765373</v>
       </c>
     </row>
     <row r="80" spans="1:7">
@@ -2220,13 +2220,13 @@
         <v>-3.836659558423335</v>
       </c>
       <c r="E80">
-        <v>-10.3785173040768</v>
+        <v>-23.62755069237609</v>
       </c>
       <c r="F80">
-        <v>1.344146077068096</v>
+        <v>-1.756445537121496</v>
       </c>
       <c r="G80">
-        <v>-0.8046557283525101</v>
+        <v>-11.05785225548656</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -2243,13 +2243,13 @@
         <v>-3.101909809410036</v>
       </c>
       <c r="E81">
-        <v>-10.56448361767579</v>
+        <v>-24.58856080391386</v>
       </c>
       <c r="F81">
-        <v>1.65189285088214</v>
+        <v>-1.848733949467388</v>
       </c>
       <c r="G81">
-        <v>-0.2599617391396039</v>
+        <v>-10.71238358628145</v>
       </c>
     </row>
     <row r="82" spans="1:7">
@@ -2266,13 +2266,13 @@
         <v>-2.336350650328801</v>
       </c>
       <c r="E82">
-        <v>-12.03167749684293</v>
+        <v>-24.20184270908083</v>
       </c>
       <c r="F82">
-        <v>1.355148452912079</v>
+        <v>-1.997714998493477</v>
       </c>
       <c r="G82">
-        <v>-1.014868749005152</v>
+        <v>-10.91582654130629</v>
       </c>
     </row>
     <row r="83" spans="1:7">
@@ -2289,13 +2289,13 @@
         <v>-1.54021050133261</v>
       </c>
       <c r="E83">
-        <v>-12.36220175771477</v>
+        <v>-25.42261967512059</v>
       </c>
       <c r="F83">
-        <v>1.398773593813112</v>
+        <v>-2.01899989890841</v>
       </c>
       <c r="G83">
-        <v>0.3523666954406127</v>
+        <v>-11.14896840036392</v>
       </c>
     </row>
     <row r="84" spans="1:7">
@@ -2312,13 +2312,13 @@
         <v>-0.7154325321820308</v>
       </c>
       <c r="E84">
-        <v>-13.40988233328534</v>
+        <v>-26.18062735384251</v>
       </c>
       <c r="F84">
-        <v>1.436979555165031</v>
+        <v>-1.849549891359146</v>
       </c>
       <c r="G84">
-        <v>0.4671300671049877</v>
+        <v>-10.70807656653486</v>
       </c>
     </row>
     <row r="85" spans="1:7">
@@ -2335,13 +2335,13 @@
         <v>0.1351353442662429</v>
       </c>
       <c r="E85">
-        <v>-14.34724475355505</v>
+        <v>-26.49677370974</v>
       </c>
       <c r="F85">
-        <v>1.03792846947962</v>
+        <v>-2.025753578343434</v>
       </c>
       <c r="G85">
-        <v>0.6557119832040316</v>
+        <v>-10.72093141486385</v>
       </c>
     </row>
     <row r="86" spans="1:7">
@@ -2358,13 +2358,13 @@
         <v>1.004226973751066</v>
       </c>
       <c r="E86">
-        <v>-16.42127679212006</v>
+        <v>-27.71844731363328</v>
       </c>
       <c r="F86">
-        <v>1.168084869277089</v>
+        <v>-2.253900871687669</v>
       </c>
       <c r="G86">
-        <v>0.8491637117913434</v>
+        <v>-10.8398230368157</v>
       </c>
     </row>
     <row r="87" spans="1:7">
@@ -2381,13 +2381,13 @@
         <v>1.882718291179257</v>
       </c>
       <c r="E87">
-        <v>-17.0524237999911</v>
+        <v>-28.07096184428637</v>
       </c>
       <c r="F87">
-        <v>1.131775869277581</v>
+        <v>-2.29651043415287</v>
       </c>
       <c r="G87">
-        <v>1.097620154513646</v>
+        <v>-10.50396819185664</v>
       </c>
     </row>
     <row r="88" spans="1:7">
@@ -2404,13 +2404,13 @@
         <v>2.760093217461863</v>
       </c>
       <c r="E88">
-        <v>-17.75398857868142</v>
+        <v>-29.09422035953357</v>
       </c>
       <c r="F88">
-        <v>1.316528307858761</v>
+        <v>-2.192998471866446</v>
       </c>
       <c r="G88">
-        <v>1.007295230020171</v>
+        <v>-10.68988842934211</v>
       </c>
     </row>
     <row r="89" spans="1:7">
@@ -2427,13 +2427,13 @@
         <v>3.620806604220227</v>
       </c>
       <c r="E89">
-        <v>-18.35533822758198</v>
+        <v>-30.2365188710204</v>
       </c>
       <c r="F89">
-        <v>1.044106433569698</v>
+        <v>-2.201383206717583</v>
       </c>
       <c r="G89">
-        <v>1.16496658241904</v>
+        <v>-10.57115902412169</v>
       </c>
     </row>
     <row r="90" spans="1:7">
@@ -2450,13 +2450,13 @@
         <v>4.447639326005682</v>
       </c>
       <c r="E90">
-        <v>-22.36369435310136</v>
+        <v>-31.28731730094525</v>
       </c>
       <c r="F90">
-        <v>1.326182101570986</v>
+        <v>-2.339136563966127</v>
       </c>
       <c r="G90">
-        <v>1.575805283842594</v>
+        <v>-11.03042769623924</v>
       </c>
     </row>
     <row r="91" spans="1:7">
@@ -2473,13 +2473,13 @@
         <v>5.21795897747709</v>
       </c>
       <c r="E91">
-        <v>-22.46654505476357</v>
+        <v>-32.45216082027927</v>
       </c>
       <c r="F91">
-        <v>1.089280621513967</v>
+        <v>-2.280054915696257</v>
       </c>
       <c r="G91">
-        <v>0.9503803311090206</v>
+        <v>-10.13732196283681</v>
       </c>
     </row>
     <row r="92" spans="1:7">
@@ -2496,13 +2496,13 @@
         <v>5.910502698445531</v>
       </c>
       <c r="E92">
-        <v>-25.05329544895103</v>
+        <v>-34.3436591285431</v>
       </c>
       <c r="F92">
-        <v>0.8972683710146523</v>
+        <v>-2.777584803328682</v>
       </c>
       <c r="G92">
-        <v>1.052345133718573</v>
+        <v>-10.82198912799564</v>
       </c>
     </row>
     <row r="93" spans="1:7">
@@ -2519,13 +2519,13 @@
         <v>6.504421394387385</v>
       </c>
       <c r="E93">
-        <v>-25.97615316697417</v>
+        <v>-34.99201433764329</v>
       </c>
       <c r="F93">
-        <v>1.033041101803102</v>
+        <v>-2.596221215792356</v>
       </c>
       <c r="G93">
-        <v>0.6118141493532956</v>
+        <v>-10.98715886604096</v>
       </c>
     </row>
     <row r="94" spans="1:7">
@@ -2542,13 +2542,13 @@
         <v>6.976013478199483</v>
       </c>
       <c r="E94">
-        <v>-29.45735189749765</v>
+        <v>-36.00955791869281</v>
       </c>
       <c r="F94">
-        <v>1.250901728739372</v>
+        <v>-2.747288922306096</v>
       </c>
       <c r="G94">
-        <v>0.8203520339630662</v>
+        <v>-10.63588018941444</v>
       </c>
     </row>
     <row r="95" spans="1:7">
@@ -2565,13 +2565,13 @@
         <v>7.315693095126392</v>
       </c>
       <c r="E95">
-        <v>-30.64758883482968</v>
+        <v>-37.8076904141035</v>
       </c>
       <c r="F95">
-        <v>0.874933929100372</v>
+        <v>-2.64126700678919</v>
       </c>
       <c r="G95">
-        <v>0.1143748871679463</v>
+        <v>-10.69325856470108</v>
       </c>
     </row>
     <row r="96" spans="1:7">
@@ -2588,13 +2588,13 @@
         <v>7.508936049310362</v>
       </c>
       <c r="E96">
-        <v>-31.68512789286007</v>
+        <v>-40.26902924912253</v>
       </c>
       <c r="F96">
-        <v>0.8037904230783394</v>
+        <v>-3.096426730135823</v>
       </c>
       <c r="G96">
-        <v>0.4312603061869844</v>
+        <v>-10.75104413708906</v>
       </c>
     </row>
     <row r="97" spans="1:7">
@@ -2611,13 +2611,13 @@
         <v>7.557897727588303</v>
       </c>
       <c r="E97">
-        <v>-34.2082826623208</v>
+        <v>-41.41522451249296</v>
       </c>
       <c r="F97">
-        <v>1.159446654000696</v>
+        <v>-3.131759913334833</v>
       </c>
       <c r="G97">
-        <v>0.4262746246048419</v>
+        <v>-11.57288044612206</v>
       </c>
     </row>
     <row r="98" spans="1:7">
@@ -2634,13 +2634,13 @@
         <v>7.446128864007064</v>
       </c>
       <c r="E98">
-        <v>-37.23067904875715</v>
+        <v>-42.96457623134427</v>
       </c>
       <c r="F98">
-        <v>0.7864029912935777</v>
+        <v>-2.958947562497606</v>
       </c>
       <c r="G98">
-        <v>-0.5003702456559382</v>
+        <v>-11.55117982011213</v>
       </c>
     </row>
     <row r="99" spans="1:7">
@@ -2657,13 +2657,13 @@
         <v>7.210537795491544</v>
       </c>
       <c r="E99">
-        <v>-39.40431713735788</v>
+        <v>-44.43741938183597</v>
       </c>
       <c r="F99">
-        <v>0.7640470118268247</v>
+        <v>-3.262538417051805</v>
       </c>
       <c r="G99">
-        <v>-0.5032570413661827</v>
+        <v>-11.53396167276239</v>
       </c>
     </row>
     <row r="100" spans="1:7">
@@ -2680,13 +2680,13 @@
         <v>6.815404670717448</v>
       </c>
       <c r="E100">
-        <v>-40.98166161828759</v>
+        <v>-46.25498355921358</v>
       </c>
       <c r="F100">
-        <v>0.7396184571182672</v>
+        <v>-3.390089601367471</v>
       </c>
       <c r="G100">
-        <v>0.074439776327718</v>
+        <v>-11.94761764843986</v>
       </c>
     </row>
     <row r="101" spans="1:7">
@@ -2703,13 +2703,13 @@
         <v>6.338435737185112</v>
       </c>
       <c r="E101">
-        <v>-43.79158653275806</v>
+        <v>-48.68104558171286</v>
       </c>
       <c r="F101">
-        <v>0.610696324750969</v>
+        <v>-3.624042093470524</v>
       </c>
       <c r="G101">
-        <v>-0.5268910259710397</v>
+        <v>-12.54612455539362</v>
       </c>
     </row>
     <row r="102" spans="1:7">
@@ -2726,13 +2726,13 @@
         <v>5.683206153406423</v>
       </c>
       <c r="E102">
-        <v>-45.84205692106116</v>
+        <v>-50.46161099432929</v>
       </c>
       <c r="F102">
-        <v>0.5963506580692871</v>
+        <v>-3.583115773567811</v>
       </c>
       <c r="G102">
-        <v>-1.417358254578664</v>
+        <v>-12.15088845509665</v>
       </c>
     </row>
   </sheetData>

</xml_diff>